<commit_message>
0402_Refactor sigma_alpha_sq to independent layers for improved Gibbs sampling
</commit_message>
<xml_diff>
--- a/data/MIDUS_wave_2_변수명세.xlsx
+++ b/data/MIDUS_wave_2_변수명세.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/todoo/Desktop/학교/대학원/Research/joint_LSIRM/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBA4CC35-80FA-DD47-8856-EF74C9BBE5FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D8AB5EB-AFAB-7243-A226-820F68362766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="16780" activeTab="1" xr2:uid="{D80E1FB4-5E45-DF4A-81BC-88625E0DBDBC}"/>
   </bookViews>

</xml_diff>

<commit_message>
0407_Add ordinal-only LSIRM implementation with C++ backend
- Introduced `lsirm_ordinal_only.R` for R interface to the ordinal-only LSIRM model.
- Added `lsirm_ordinal_only.cpp` for C++ implementation of the MCMC algorithm.
- Created `test_ordinal_only_result.R` for testing and visualizing results of the ordinal-only model.
- Implemented data preprocessing and MCMC settings for combining datasets from Wave 2 and Refresher 1.
- Added functions for generating trace plots and biplots to visualize latent spaces.
- Included acceptance rate reporting for MCMC parameters.
</commit_message>
<xml_diff>
--- a/data/MIDUS_wave_2_변수명세.xlsx
+++ b/data/MIDUS_wave_2_변수명세.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/todoo/Desktop/학교/대학원/Research/joint_LSIRM/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{619326D5-C70D-4A49-B4DB-0036CEFDA419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8E0F49E-8970-6B4A-AE1A-C5BA2B4B8C4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="0" windowWidth="28800" windowHeight="16720" xr2:uid="{D80E1FB4-5E45-DF4A-81BC-88625E0DBDBC}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="16680" xr2:uid="{D80E1FB4-5E45-DF4A-81BC-88625E0DBDBC}"/>
   </bookViews>
   <sheets>
-    <sheet name="변수list" sheetId="2" r:id="rId1"/>
+    <sheet name="wave_2_변수list" sheetId="2" r:id="rId1"/>
+    <sheet name="refresher_1_변수list" sheetId="4" r:id="rId2"/>
+    <sheet name="wave 정리" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1128" uniqueCount="394">
   <si>
     <t>변수명</t>
   </si>
@@ -813,13 +815,418 @@
   </si>
   <si>
     <t>MASQ 불안/각성 관련 변수 추가</t>
+  </si>
+  <si>
+    <t>MIDUS wave 2</t>
+  </si>
+  <si>
+    <t>survey</t>
+  </si>
+  <si>
+    <t>biomarker</t>
+  </si>
+  <si>
+    <t>cognitive</t>
+  </si>
+  <si>
+    <t>refresher 1</t>
+  </si>
+  <si>
+    <t>수집 시기</t>
+  </si>
+  <si>
+    <t>2004 - 2006</t>
+  </si>
+  <si>
+    <t>2004 - 2009</t>
+  </si>
+  <si>
+    <t>2011 - 2014</t>
+  </si>
+  <si>
+    <t>2012 - 2016</t>
+  </si>
+  <si>
+    <t>보류(NA 너무많음)</t>
+  </si>
+  <si>
+    <t>M2P1 (ICPSR 36532)</t>
+  </si>
+  <si>
+    <t>M2P4 (ICPSR 36901)</t>
+  </si>
+  <si>
+    <t>M2P4 (ICPSR 37081)</t>
+  </si>
+  <si>
+    <t>RA1PA60</t>
+  </si>
+  <si>
+    <t>RA1PA61</t>
+  </si>
+  <si>
+    <t>RA1PA62</t>
+  </si>
+  <si>
+    <t>RA1PA72</t>
+  </si>
+  <si>
+    <t>RA1PA73</t>
+  </si>
+  <si>
+    <t>RA1PA74</t>
+  </si>
+  <si>
+    <t>RA4S4</t>
+  </si>
+  <si>
+    <t>RA4S5</t>
+  </si>
+  <si>
+    <t>RA3TCOMPZ3</t>
+  </si>
+  <si>
+    <t>RA3TEMZ3</t>
+  </si>
+  <si>
+    <t>RA3TEFZ3</t>
+  </si>
+  <si>
+    <t>RA3TWLF</t>
+  </si>
+  <si>
+    <t>RA3TSMXNS</t>
+  </si>
+  <si>
+    <t>RA3TSMXRS</t>
+  </si>
+  <si>
+    <t>RA4P2A</t>
+  </si>
+  <si>
+    <t>RA4PWHR</t>
+  </si>
+  <si>
+    <t>RA4Q3A</t>
+  </si>
+  <si>
+    <t>RA4Q3C</t>
+  </si>
+  <si>
+    <t>RA4Q3D</t>
+  </si>
+  <si>
+    <t>RA4Q3E</t>
+  </si>
+  <si>
+    <t>RA4Q3F</t>
+  </si>
+  <si>
+    <t>RA4Q3G</t>
+  </si>
+  <si>
+    <t>RA4Q3H</t>
+  </si>
+  <si>
+    <t>RA4Q3I</t>
+  </si>
+  <si>
+    <t>RA4Q3J</t>
+  </si>
+  <si>
+    <t>RA4Q3K</t>
+  </si>
+  <si>
+    <t>RA4Q3L</t>
+  </si>
+  <si>
+    <t>RA4Q3M</t>
+  </si>
+  <si>
+    <t>RA4Q3N</t>
+  </si>
+  <si>
+    <t>RA4Q3O</t>
+  </si>
+  <si>
+    <t>RA4Q3P</t>
+  </si>
+  <si>
+    <t>RA4Q3Q</t>
+  </si>
+  <si>
+    <t>RA4Q3R</t>
+  </si>
+  <si>
+    <t>RA4Q3S</t>
+  </si>
+  <si>
+    <t>RA4Q3T</t>
+  </si>
+  <si>
+    <t>RA4Q1D</t>
+  </si>
+  <si>
+    <t>RA4Q1H</t>
+  </si>
+  <si>
+    <t>RA4Q1K</t>
+  </si>
+  <si>
+    <t>RA4Q1N</t>
+  </si>
+  <si>
+    <t>RA4Q1P</t>
+  </si>
+  <si>
+    <t>RA4Q1T</t>
+  </si>
+  <si>
+    <t>RA4Q1Z</t>
+  </si>
+  <si>
+    <t>RA4Q1FF</t>
+  </si>
+  <si>
+    <t>RA4Q1II</t>
+  </si>
+  <si>
+    <t>RA4Q1CCC</t>
+  </si>
+  <si>
+    <t>RA4Q1GGG</t>
+  </si>
+  <si>
+    <t>RA4Q1F</t>
+  </si>
+  <si>
+    <t>RA4Q1M</t>
+  </si>
+  <si>
+    <t>RA4Q1Q</t>
+  </si>
+  <si>
+    <t>RA4Q1S</t>
+  </si>
+  <si>
+    <t>RA4Q1X</t>
+  </si>
+  <si>
+    <t>RA4Q1DD</t>
+  </si>
+  <si>
+    <t>RA4Q1KK</t>
+  </si>
+  <si>
+    <t>RA4Q1NN</t>
+  </si>
+  <si>
+    <t>RA4Q1PP</t>
+  </si>
+  <si>
+    <t>RA4Q1RR</t>
+  </si>
+  <si>
+    <t>RA4Q1TT</t>
+  </si>
+  <si>
+    <t>RA4Q1VV</t>
+  </si>
+  <si>
+    <t>RA4Q1ZZ</t>
+  </si>
+  <si>
+    <t>RA4Q1JJJ</t>
+  </si>
+  <si>
+    <t>RA4BSCL4A</t>
+  </si>
+  <si>
+    <t>RA4BSCLAV</t>
+  </si>
+  <si>
+    <t>RA4BNE12</t>
+  </si>
+  <si>
+    <t>RA4BIL6</t>
+  </si>
+  <si>
+    <t>RA4BFGN</t>
+  </si>
+  <si>
+    <t>RA4BCRP</t>
+  </si>
+  <si>
+    <t>RA4H41</t>
+  </si>
+  <si>
+    <t>RA4Q3B</t>
+  </si>
+  <si>
+    <t>RA4Q1B</t>
+  </si>
+  <si>
+    <t>RA4Q1BB</t>
+  </si>
+  <si>
+    <t>RA4Q1BBB</t>
+  </si>
+  <si>
+    <t>wave 2 에는 있으나 refresher 에는 없음</t>
+  </si>
+  <si>
+    <t>wave 2 와 refresher 에 표기가 다름</t>
+  </si>
+  <si>
+    <t>오류 - wave 2 포함해서 확인 필요</t>
+  </si>
+  <si>
+    <t>제거 - refresher_1 에 없음</t>
+  </si>
+  <si>
+    <t>RA4H38</t>
+  </si>
+  <si>
+    <t>RA4H56</t>
+  </si>
+  <si>
+    <t>RA4H49</t>
+  </si>
+  <si>
+    <t>B3TSPN</t>
+  </si>
+  <si>
+    <t>B3TSPR</t>
+  </si>
+  <si>
+    <t>B3TSMN</t>
+  </si>
+  <si>
+    <t>B3TSMR</t>
+  </si>
+  <si>
+    <t>B3TSMXBS</t>
+  </si>
+  <si>
+    <t>B3TSMXNO</t>
+  </si>
+  <si>
+    <t>B3TSMXRO</t>
+  </si>
+  <si>
+    <t>B3TCTFLR</t>
+  </si>
+  <si>
+    <t>B3TCTFLI</t>
+  </si>
+  <si>
+    <t>0.5로 나눠서 integer 화 / 문제 상한 20이므로 reverse coding 으로 틀린 문제 수로 해석</t>
+  </si>
+  <si>
+    <t>B3TSMXNS, B3TSMXRS 의 상위지표로 두개 대체 가능</t>
+  </si>
+  <si>
+    <t>zero - inflated 가능성</t>
+  </si>
+  <si>
+    <t>Verbal Fluency</t>
+  </si>
+  <si>
+    <t>Task Switching</t>
+  </si>
+  <si>
+    <t>Executive Function / Processing Speed</t>
+  </si>
+  <si>
+    <t>보류(패턴을 해침)</t>
+  </si>
+  <si>
+    <t>RA3TSPN</t>
+  </si>
+  <si>
+    <t>RA3TSPR</t>
+  </si>
+  <si>
+    <t>RA3TSMN</t>
+  </si>
+  <si>
+    <t>RA3TSMR</t>
+  </si>
+  <si>
+    <t>RA3TSMXBS</t>
+  </si>
+  <si>
+    <t>RA3TSMXNO</t>
+  </si>
+  <si>
+    <t>RA3TSMXRO</t>
+  </si>
+  <si>
+    <t>RA3TCTFLR</t>
+  </si>
+  <si>
+    <t>RA3TCTFLI</t>
+  </si>
+  <si>
+    <t>SGST Normal single-task 정확도 (정답 비율, 0~1)</t>
+  </si>
+  <si>
+    <t>기본 과제 수행 정확성</t>
+  </si>
+  <si>
+    <t>SGST Reverse single-task 정확도 (정답 비율, 0~1)</t>
+  </si>
+  <si>
+    <t>역규칙 과제 수행 정확성 (inhibitory control)</t>
+  </si>
+  <si>
+    <t>SGST Normal single-task 정답 trial median RT (초)</t>
+  </si>
+  <si>
+    <t>기본 인지 처리 속도 baseline</t>
+  </si>
+  <si>
+    <t>SGST Reverse single-task 정답 trial median RT (초)</t>
+  </si>
+  <si>
+    <t>역규칙 처리 속도 (inhibition cost 반영)</t>
+  </si>
+  <si>
+    <t>SGST Mixed block 전체 switch trial median RT (초)</t>
+  </si>
+  <si>
+    <t>규칙 전환 시 반응 속도 (cognitive flexibility)</t>
+  </si>
+  <si>
+    <t>SGST Mixed block normal non-switch trial median RT (초)</t>
+  </si>
+  <si>
+    <t>Mixed block 내 규칙 유지 속도 (normal, mixing cost 포함)</t>
+  </si>
+  <si>
+    <t>SGST Mixed block reverse non-switch trial median RT (초)</t>
+  </si>
+  <si>
+    <t>Mixed block 내 규칙 유지 속도 (reverse, mixing cost 포함)</t>
+  </si>
+  <si>
+    <t>Category fluency 반복 수 (같은 단어 재언급 횟수)</t>
+  </si>
+  <si>
+    <t>자기 모니터링 실패 빈도</t>
+  </si>
+  <si>
+    <t>Category fluency 침입 오류 수 (범주 밖 단어 응답 횟수)</t>
+  </si>
+  <si>
+    <t>Semantic boundary 통제 실패 / executive monitoring</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -858,8 +1265,43 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -874,6 +1316,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -904,7 +1364,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -915,6 +1375,19 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1249,14 +1722,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87BBB518-99D5-8443-BE8B-68691D1BDDA9}">
-  <dimension ref="C3:K84"/>
+  <dimension ref="C3:K108"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="19.1640625" customWidth="1"/>
+    <col min="3" max="3" width="32.5" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="106.6640625" customWidth="1"/>
-    <col min="6" max="6" width="19.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.5" customWidth="1"/>
+    <col min="5" max="5" width="25.1640625" customWidth="1"/>
+    <col min="6" max="6" width="10.1640625" customWidth="1"/>
+    <col min="7" max="7" width="18.33203125" customWidth="1"/>
     <col min="8" max="8" width="38.1640625" customWidth="1"/>
     <col min="9" max="9" width="15.33203125" customWidth="1"/>
     <col min="10" max="10" width="38.6640625" customWidth="1"/>
@@ -1472,6 +1945,9 @@
       <c r="H13" t="s">
         <v>63</v>
       </c>
+      <c r="I13" s="6" t="s">
+        <v>347</v>
+      </c>
     </row>
     <row r="14" spans="3:11" x14ac:dyDescent="0.2">
       <c r="C14" t="s">
@@ -1534,7 +2010,7 @@
       </c>
       <c r="K16" s="3"/>
     </row>
-    <row r="17" spans="3:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C17" t="s">
         <v>67</v>
       </c>
@@ -1554,7 +2030,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="3:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C18" t="s">
         <v>68</v>
       </c>
@@ -1574,7 +2050,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="3:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C19" t="s">
         <v>69</v>
       </c>
@@ -1594,7 +2070,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="3:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C20" t="s">
         <v>70</v>
       </c>
@@ -1614,7 +2090,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="3:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C21" t="s">
         <v>70</v>
       </c>
@@ -1634,7 +2110,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="22" spans="3:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C22" t="s">
         <v>73</v>
       </c>
@@ -1653,8 +2129,11 @@
       <c r="H22" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="23" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="I22" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="23" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C23" t="s">
         <v>40</v>
       </c>
@@ -1673,8 +2152,11 @@
       <c r="H23" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="24" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="I23" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="24" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C24" t="s">
         <v>77</v>
       </c>
@@ -1694,7 +2176,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="25" spans="3:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C25" t="s">
         <v>77</v>
       </c>
@@ -1714,7 +2196,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="26" spans="3:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C26" t="s">
         <v>77</v>
       </c>
@@ -1734,7 +2216,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="27" spans="3:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C27" t="s">
         <v>144</v>
       </c>
@@ -1753,8 +2235,11 @@
       <c r="H27" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="28" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="I27" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="28" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C28" t="s">
         <v>148</v>
       </c>
@@ -1773,8 +2258,11 @@
       <c r="H28" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="29" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="I28" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="29" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C29" t="s">
         <v>152</v>
       </c>
@@ -1793,8 +2281,11 @@
       <c r="H29" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="30" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="I29" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="30" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C30" t="s">
         <v>156</v>
       </c>
@@ -1813,8 +2304,11 @@
       <c r="H30" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="31" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="I30" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="31" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C31" t="s">
         <v>161</v>
       </c>
@@ -1833,8 +2327,11 @@
       <c r="H31" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="32" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="I31" s="6" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="32" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C32" t="s">
         <v>62</v>
       </c>
@@ -1852,6 +2349,9 @@
       </c>
       <c r="H32" t="s">
         <v>169</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="33" spans="3:10" x14ac:dyDescent="0.2">
@@ -2314,20 +2814,80 @@
         <v>256</v>
       </c>
     </row>
-    <row r="56" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C56" t="s">
+    <row r="53" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C53" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="57" spans="3:10" ht="42" x14ac:dyDescent="0.2">
+    <row r="54" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C54" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H54" s="4" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="55" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C55" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G55" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H55" s="4" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="56" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C56" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H56" s="4" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="57" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C57" s="4" t="s">
         <v>241</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="F57" s="4" t="s">
         <v>61</v>
@@ -2339,15 +2899,15 @@
         <v>242</v>
       </c>
     </row>
-    <row r="58" spans="3:10" ht="42" x14ac:dyDescent="0.2">
+    <row r="58" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C58" s="4" t="s">
         <v>241</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="F58" s="4" t="s">
         <v>61</v>
@@ -2356,18 +2916,18 @@
         <v>84</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="59" spans="3:10" ht="42" x14ac:dyDescent="0.2">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="59" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C59" s="4" t="s">
         <v>241</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>5</v>
+        <v>102</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>6</v>
+        <v>103</v>
       </c>
       <c r="F59" s="4" t="s">
         <v>61</v>
@@ -2376,18 +2936,18 @@
         <v>84</v>
       </c>
       <c r="H59" s="4" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="60" spans="3:10" ht="42" x14ac:dyDescent="0.2">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="60" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C60" s="4" t="s">
         <v>241</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="F60" s="4" t="s">
         <v>61</v>
@@ -2396,18 +2956,18 @@
         <v>84</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="61" spans="3:10" ht="42" x14ac:dyDescent="0.2">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="61" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C61" s="4" t="s">
         <v>241</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>96</v>
+        <v>112</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
       <c r="F61" s="4" t="s">
         <v>61</v>
@@ -2416,18 +2976,18 @@
         <v>84</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="62" spans="3:10" ht="42" x14ac:dyDescent="0.2">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="62" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C62" s="4" t="s">
         <v>241</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="F62" s="4" t="s">
         <v>61</v>
@@ -2439,15 +2999,15 @@
         <v>243</v>
       </c>
     </row>
-    <row r="63" spans="3:10" ht="42" x14ac:dyDescent="0.2">
+    <row r="63" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C63" s="4" t="s">
         <v>241</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>107</v>
+        <v>132</v>
       </c>
       <c r="F63" s="4" t="s">
         <v>61</v>
@@ -2459,15 +3019,15 @@
         <v>91</v>
       </c>
     </row>
-    <row r="64" spans="3:10" ht="42" x14ac:dyDescent="0.2">
+    <row r="64" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C64" s="4" t="s">
         <v>241</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="F64" s="4" t="s">
         <v>61</v>
@@ -2476,78 +3036,78 @@
         <v>84</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="65" spans="3:8" ht="42" x14ac:dyDescent="0.2">
-      <c r="C65" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="D65" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="E65" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="F65" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="G65" s="4" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="65" spans="3:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C65" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D65" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="E65" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="F65" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="G65" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="H65" s="4" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="66" spans="3:8" ht="42" x14ac:dyDescent="0.2">
-      <c r="C66" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="D66" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="E66" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="F66" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="G66" s="4" t="s">
+      <c r="H65" s="5" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="66" spans="3:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C66" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D66" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E66" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F66" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="G66" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="H66" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="67" spans="3:8" ht="42" x14ac:dyDescent="0.2">
-      <c r="C67" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="D67" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="E67" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="F67" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="G67" s="4" t="s">
+      <c r="H66" s="5" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="67" spans="3:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C67" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D67" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="E67" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="F67" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="G67" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="H67" s="4" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="68" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="H67" s="5" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="68" spans="3:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C68" s="5" t="s">
         <v>246</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="F68" s="5" t="s">
         <v>61</v>
@@ -2556,18 +3116,18 @@
         <v>84</v>
       </c>
       <c r="H68" s="5" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="69" spans="3:8" x14ac:dyDescent="0.2">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="69" spans="3:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C69" s="5" t="s">
         <v>246</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="F69" s="5" t="s">
         <v>61</v>
@@ -2579,15 +3139,15 @@
         <v>248</v>
       </c>
     </row>
-    <row r="70" spans="3:8" x14ac:dyDescent="0.2">
+    <row r="70" spans="3:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C70" s="5" t="s">
         <v>246</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="F70" s="5" t="s">
         <v>61</v>
@@ -2596,18 +3156,18 @@
         <v>84</v>
       </c>
       <c r="H70" s="5" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="71" spans="3:8" x14ac:dyDescent="0.2">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="71" spans="3:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C71" s="5" t="s">
         <v>246</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="F71" s="5" t="s">
         <v>61</v>
@@ -2616,18 +3176,18 @@
         <v>84</v>
       </c>
       <c r="H71" s="5" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="72" spans="3:8" x14ac:dyDescent="0.2">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="72" spans="3:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C72" s="5" t="s">
         <v>246</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="F72" s="5" t="s">
         <v>61</v>
@@ -2636,18 +3196,18 @@
         <v>84</v>
       </c>
       <c r="H72" s="5" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="73" spans="3:8" x14ac:dyDescent="0.2">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="73" spans="3:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C73" s="5" t="s">
         <v>246</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="F73" s="5" t="s">
         <v>61</v>
@@ -2659,15 +3219,15 @@
         <v>248</v>
       </c>
     </row>
-    <row r="74" spans="3:8" x14ac:dyDescent="0.2">
+    <row r="74" spans="3:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C74" s="5" t="s">
         <v>246</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="F74" s="5" t="s">
         <v>61</v>
@@ -2676,18 +3236,18 @@
         <v>84</v>
       </c>
       <c r="H74" s="5" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="75" spans="3:8" x14ac:dyDescent="0.2">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="75" spans="3:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C75" s="5" t="s">
         <v>246</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="F75" s="5" t="s">
         <v>61</v>
@@ -2696,18 +3256,18 @@
         <v>84</v>
       </c>
       <c r="H75" s="5" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="76" spans="3:8" x14ac:dyDescent="0.2">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="76" spans="3:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C76" s="5" t="s">
         <v>246</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="F76" s="5" t="s">
         <v>61</v>
@@ -2716,18 +3276,18 @@
         <v>84</v>
       </c>
       <c r="H76" s="5" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="77" spans="3:8" x14ac:dyDescent="0.2">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="77" spans="3:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C77" s="5" t="s">
         <v>246</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="E77" s="5" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="F77" s="5" t="s">
         <v>61</v>
@@ -2736,18 +3296,18 @@
         <v>84</v>
       </c>
       <c r="H77" s="5" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="78" spans="3:8" x14ac:dyDescent="0.2">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="78" spans="3:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C78" s="5" t="s">
         <v>246</v>
       </c>
       <c r="D78" s="5" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="E78" s="5" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="F78" s="5" t="s">
         <v>61</v>
@@ -2756,18 +3316,18 @@
         <v>84</v>
       </c>
       <c r="H78" s="5" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="79" spans="3:8" x14ac:dyDescent="0.2">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="79" spans="3:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C79" s="5" t="s">
         <v>246</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="E79" s="5" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="F79" s="5" t="s">
         <v>61</v>
@@ -2776,18 +3336,18 @@
         <v>84</v>
       </c>
       <c r="H79" s="5" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="80" spans="3:8" x14ac:dyDescent="0.2">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="80" spans="3:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C80" s="5" t="s">
         <v>246</v>
       </c>
       <c r="D80" s="5" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>125</v>
+        <v>254</v>
       </c>
       <c r="F80" s="5" t="s">
         <v>61</v>
@@ -2796,18 +3356,18 @@
         <v>84</v>
       </c>
       <c r="H80" s="5" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="81" spans="3:8" x14ac:dyDescent="0.2">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="81" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C81" s="5" t="s">
         <v>246</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="F81" s="5" t="s">
         <v>61</v>
@@ -2816,72 +3376,2304 @@
         <v>84</v>
       </c>
       <c r="H81" s="5" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="82" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="C82" s="5" t="s">
-        <v>246</v>
-      </c>
-      <c r="D82" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="E82" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="F82" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="G82" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="H82" s="5" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="83" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="C83" s="5" t="s">
-        <v>246</v>
-      </c>
-      <c r="D83" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="E83" s="5" t="s">
-        <v>254</v>
-      </c>
-      <c r="F83" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="G83" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="H83" s="5" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="84" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="C84" s="5" t="s">
-        <v>246</v>
-      </c>
-      <c r="D84" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="E84" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="F84" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="G84" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="H84" s="5" t="s">
         <v>248</v>
       </c>
+    </row>
+    <row r="82" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="83" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="84" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="89" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C89" t="s">
+        <v>365</v>
+      </c>
+      <c r="D89" t="s">
+        <v>351</v>
+      </c>
+      <c r="E89" s="18" t="s">
+        <v>376</v>
+      </c>
+      <c r="F89" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G89" t="s">
+        <v>140</v>
+      </c>
+      <c r="H89" s="18" t="s">
+        <v>377</v>
+      </c>
+      <c r="J89" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="90" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C90" t="s">
+        <v>365</v>
+      </c>
+      <c r="D90" t="s">
+        <v>352</v>
+      </c>
+      <c r="E90" s="18" t="s">
+        <v>378</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G90" t="s">
+        <v>140</v>
+      </c>
+      <c r="H90" s="18" t="s">
+        <v>379</v>
+      </c>
+      <c r="J90" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="91" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C91" t="s">
+        <v>365</v>
+      </c>
+      <c r="D91" t="s">
+        <v>353</v>
+      </c>
+      <c r="E91" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G91" t="s">
+        <v>34</v>
+      </c>
+      <c r="H91" s="18" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="92" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C92" t="s">
+        <v>365</v>
+      </c>
+      <c r="D92" t="s">
+        <v>354</v>
+      </c>
+      <c r="E92" s="18" t="s">
+        <v>382</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G92" t="s">
+        <v>34</v>
+      </c>
+      <c r="H92" s="18" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="93" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C93" t="s">
+        <v>364</v>
+      </c>
+      <c r="D93" t="s">
+        <v>355</v>
+      </c>
+      <c r="E93" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G93" t="s">
+        <v>34</v>
+      </c>
+      <c r="H93" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="J93" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="94" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C94" t="s">
+        <v>364</v>
+      </c>
+      <c r="D94" t="s">
+        <v>356</v>
+      </c>
+      <c r="E94" s="18" t="s">
+        <v>386</v>
+      </c>
+      <c r="F94" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G94" t="s">
+        <v>34</v>
+      </c>
+      <c r="H94" s="18" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="95" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C95" t="s">
+        <v>364</v>
+      </c>
+      <c r="D95" t="s">
+        <v>357</v>
+      </c>
+      <c r="E95" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="F95" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G95" t="s">
+        <v>34</v>
+      </c>
+      <c r="H95" s="18" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="96" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C96" t="s">
+        <v>363</v>
+      </c>
+      <c r="D96" t="s">
+        <v>358</v>
+      </c>
+      <c r="E96" s="18" t="s">
+        <v>390</v>
+      </c>
+      <c r="F96" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G96" t="s">
+        <v>140</v>
+      </c>
+      <c r="H96" s="18" t="s">
+        <v>391</v>
+      </c>
+      <c r="J96" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="97" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C97" t="s">
+        <v>363</v>
+      </c>
+      <c r="D97" t="s">
+        <v>359</v>
+      </c>
+      <c r="E97" s="18" t="s">
+        <v>392</v>
+      </c>
+      <c r="F97" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G97" t="s">
+        <v>140</v>
+      </c>
+      <c r="H97" s="18" t="s">
+        <v>393</v>
+      </c>
+      <c r="J97" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="99" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C99" s="17"/>
+      <c r="D99" s="17"/>
+      <c r="E99" s="17"/>
+      <c r="F99" s="17"/>
+      <c r="G99" s="17"/>
+      <c r="H99" s="17"/>
+      <c r="I99" s="17"/>
+    </row>
+    <row r="100" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C100" s="18"/>
+      <c r="D100" s="18"/>
+      <c r="F100" s="18"/>
+      <c r="G100" s="18"/>
+      <c r="I100" s="18"/>
+    </row>
+    <row r="101" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C101" t="s">
+        <v>363</v>
+      </c>
+      <c r="D101" t="s">
+        <v>358</v>
+      </c>
+      <c r="F101" s="18"/>
+      <c r="G101" s="18"/>
+      <c r="I101" s="18"/>
+    </row>
+    <row r="102" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C102" t="s">
+        <v>363</v>
+      </c>
+      <c r="D102" t="s">
+        <v>359</v>
+      </c>
+      <c r="F102" s="18"/>
+      <c r="G102" s="18"/>
+      <c r="I102" s="18"/>
+    </row>
+    <row r="103" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C103" t="s">
+        <v>365</v>
+      </c>
+      <c r="D103" t="s">
+        <v>351</v>
+      </c>
+      <c r="F103" s="18"/>
+      <c r="G103" s="18"/>
+      <c r="I103" s="18"/>
+    </row>
+    <row r="104" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C104" t="s">
+        <v>365</v>
+      </c>
+      <c r="D104" t="s">
+        <v>352</v>
+      </c>
+      <c r="F104" s="18"/>
+      <c r="G104" s="18"/>
+      <c r="I104" s="18"/>
+    </row>
+    <row r="105" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C105" s="18"/>
+      <c r="D105" s="18"/>
+      <c r="F105" s="18"/>
+      <c r="G105" s="18"/>
+      <c r="I105" s="18"/>
+    </row>
+    <row r="106" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C106" s="18"/>
+      <c r="D106" s="18"/>
+      <c r="F106" s="18"/>
+      <c r="G106" s="18"/>
+      <c r="I106" s="18"/>
+    </row>
+    <row r="107" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C107" s="18"/>
+      <c r="D107" s="18"/>
+      <c r="F107" s="18"/>
+      <c r="G107" s="18"/>
+      <c r="I107" s="18"/>
+    </row>
+    <row r="108" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C108" s="18"/>
+      <c r="D108" s="18"/>
+      <c r="F108" s="18"/>
+      <c r="G108" s="18"/>
+      <c r="I108" s="18"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0011D2F9-D328-BC45-B53A-0F0FF3C21D15}">
+  <dimension ref="C3:J103"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="35" customWidth="1"/>
+    <col min="4" max="4" width="23" customWidth="1"/>
+    <col min="5" max="5" width="79.6640625" customWidth="1"/>
+    <col min="6" max="6" width="18.33203125" customWidth="1"/>
+    <col min="7" max="7" width="22.6640625" customWidth="1"/>
+    <col min="8" max="8" width="35.83203125" customWidth="1"/>
+    <col min="9" max="9" width="17.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C3" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+    </row>
+    <row r="4" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C4" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="5" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C5" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
+    </row>
+    <row r="6" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C6" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I6" s="6"/>
+      <c r="J6" s="6"/>
+    </row>
+    <row r="7" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C7" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+    </row>
+    <row r="8" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C8" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6"/>
+    </row>
+    <row r="9" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C9" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6"/>
+    </row>
+    <row r="10" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C10" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
+    </row>
+    <row r="11" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C11" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+    </row>
+    <row r="12" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C12" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6"/>
+    </row>
+    <row r="13" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C13" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>333</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="H13" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="J13" s="6"/>
+    </row>
+    <row r="14" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C14" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>271</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="I14" s="6"/>
+      <c r="J14" s="6"/>
+    </row>
+    <row r="15" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C15" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>335</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>271</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="I15" s="6"/>
+      <c r="J15" s="6"/>
+    </row>
+    <row r="16" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C16" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="I16" s="6"/>
+      <c r="J16" s="6"/>
+    </row>
+    <row r="17" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C17" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I17" s="6"/>
+      <c r="J17" s="6"/>
+    </row>
+    <row r="18" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C18" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I18" s="6"/>
+      <c r="J18" s="6"/>
+    </row>
+    <row r="19" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C19" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+    </row>
+    <row r="20" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C20" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="I20" s="6"/>
+      <c r="J20" s="6"/>
+    </row>
+    <row r="21" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C21" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6"/>
+    </row>
+    <row r="22" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C22" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="I22" s="6"/>
+      <c r="J22" s="6"/>
+    </row>
+    <row r="23" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C23" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="I23" s="6"/>
+      <c r="J23" s="6"/>
+    </row>
+    <row r="24" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C24" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="I24" s="6"/>
+      <c r="J24" s="6"/>
+    </row>
+    <row r="25" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C25" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="I25" s="6"/>
+      <c r="J25" s="6"/>
+    </row>
+    <row r="26" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C26" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="I26" s="6"/>
+      <c r="J26" s="6"/>
+    </row>
+    <row r="27" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C27" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>348</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>271</v>
+      </c>
+      <c r="G27" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="H27" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="I27" s="6"/>
+      <c r="J27" s="6"/>
+    </row>
+    <row r="28" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C28" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>271</v>
+      </c>
+      <c r="G28" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="I28" s="6"/>
+      <c r="J28" s="6"/>
+    </row>
+    <row r="29" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C29" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>350</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>271</v>
+      </c>
+      <c r="G29" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="H29" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="I29" s="6"/>
+      <c r="J29" s="6"/>
+    </row>
+    <row r="30" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C30" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>349</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>271</v>
+      </c>
+      <c r="G30" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="H30" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="I30" s="6"/>
+      <c r="J30" s="6"/>
+    </row>
+    <row r="31" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C31" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="J31" s="6"/>
+    </row>
+    <row r="32" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C32" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="J32" s="6"/>
+    </row>
+    <row r="33" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C33" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="I33" s="6"/>
+      <c r="J33" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="34" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C34" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H34" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="I34" s="6"/>
+      <c r="J34" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="35" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C35" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="I35" s="6"/>
+      <c r="J35" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="36" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C36" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G36" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="I36" s="6"/>
+      <c r="J36" s="6" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="37" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C37" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="I37" s="6"/>
+      <c r="J37" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="38" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C38" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="I38" s="6"/>
+      <c r="J38" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="39" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C39" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="F39" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="I39" s="6"/>
+      <c r="J39" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="40" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C40" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G40" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="I40" s="6"/>
+      <c r="J40" s="6" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="41" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C41" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="I41" s="6"/>
+      <c r="J41" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="42" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C42" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="F42" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G42" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H42" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="I42" s="6"/>
+      <c r="J42" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="43" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C43" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="F43" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G43" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H43" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="I43" s="6"/>
+      <c r="J43" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="44" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C44" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G44" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H44" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="I44" s="6"/>
+      <c r="J44" s="6" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="45" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C45" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="E45" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="F45" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="I45" s="6"/>
+      <c r="J45" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="46" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C46" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="E46" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="F46" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G46" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H46" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="I46" s="6"/>
+      <c r="J46" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="47" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C47" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>302</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="F47" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G47" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H47" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="I47" s="6"/>
+      <c r="J47" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="48" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C48" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="F48" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G48" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H48" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="I48" s="6"/>
+      <c r="J48" s="6" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="49" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C49" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>304</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="F49" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G49" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H49" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="I49" s="6"/>
+      <c r="J49" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="50" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C50" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="F50" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G50" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H50" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="I50" s="6"/>
+      <c r="J50" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="51" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C51" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="E51" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="F51" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G51" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H51" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="I51" s="6"/>
+      <c r="J51" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="52" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C52" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="E52" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="F52" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="G52" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H52" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="I52" s="6"/>
+      <c r="J52" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="53" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C53" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="54" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C54" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H54" s="4" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="55" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C55" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="G55" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H55" s="4" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="56" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C56" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H56" s="4" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="57" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C57" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="G57" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H57" s="4" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="58" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C58" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="G58" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H58" s="4" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="59" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C59" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="G59" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H59" s="4" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="60" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C60" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="E60" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="F60" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="G60" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H60" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="61" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C61" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="E61" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="G61" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H61" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="62" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C62" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="E62" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="F62" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="G62" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H62" s="4" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="63" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C63" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="E63" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="F63" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="G63" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H63" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="64" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C64" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="E64" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="F64" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="G64" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H64" s="4" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="65" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C65" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D65" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="E65" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="F65" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G65" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H65" s="5" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="66" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C66" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D66" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="E66" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F66" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G66" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H66" s="5" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="67" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C67" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D67" s="5" t="s">
+        <v>320</v>
+      </c>
+      <c r="E67" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="F67" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G67" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H67" s="5" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="68" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C68" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D68" s="5" t="s">
+        <v>321</v>
+      </c>
+      <c r="E68" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="F68" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G68" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H68" s="5" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="69" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C69" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D69" s="5" t="s">
+        <v>322</v>
+      </c>
+      <c r="E69" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="F69" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G69" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H69" s="5" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="70" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C70" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D70" s="5" t="s">
+        <v>323</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="F70" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G70" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H70" s="5" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="71" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C71" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D71" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="E71" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="F71" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G71" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H71" s="5" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="72" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C72" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D72" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="E72" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="F72" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G72" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H72" s="5" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="73" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C73" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D73" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="E73" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="F73" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G73" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H73" s="5" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="74" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C74" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D74" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="E74" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="F74" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G74" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H74" s="5" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="75" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C75" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>327</v>
+      </c>
+      <c r="E75" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="F75" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G75" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H75" s="5" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="76" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C76" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D76" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="E76" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="F76" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G76" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H76" s="5" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="77" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C77" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D77" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="E77" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="F77" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G77" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H77" s="5" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="78" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C78" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D78" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="E78" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="F78" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G78" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H78" s="5" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="79" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C79" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D79" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="E79" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="F79" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G79" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H79" s="5" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="80" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="C80" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D80" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="E80" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="F80" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G80" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H80" s="5" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="81" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C81" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D81" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="E81" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="F81" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G81" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H81" s="5" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="85" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C85" s="14"/>
+      <c r="D85" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="86" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C86" s="15"/>
+      <c r="D86" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="87" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C87" s="16"/>
+      <c r="D87" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="95" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C95" t="s">
+        <v>365</v>
+      </c>
+      <c r="D95" t="s">
+        <v>367</v>
+      </c>
+      <c r="E95" s="18" t="s">
+        <v>376</v>
+      </c>
+      <c r="F95" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G95" t="s">
+        <v>140</v>
+      </c>
+      <c r="H95" s="18" t="s">
+        <v>377</v>
+      </c>
+      <c r="J95" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="96" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C96" t="s">
+        <v>365</v>
+      </c>
+      <c r="D96" t="s">
+        <v>368</v>
+      </c>
+      <c r="E96" s="18" t="s">
+        <v>378</v>
+      </c>
+      <c r="F96" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G96" t="s">
+        <v>140</v>
+      </c>
+      <c r="H96" s="18" t="s">
+        <v>379</v>
+      </c>
+      <c r="J96" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="97" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C97" t="s">
+        <v>365</v>
+      </c>
+      <c r="D97" t="s">
+        <v>369</v>
+      </c>
+      <c r="E97" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="F97" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G97" t="s">
+        <v>34</v>
+      </c>
+      <c r="H97" s="18" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="98" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C98" t="s">
+        <v>365</v>
+      </c>
+      <c r="D98" t="s">
+        <v>370</v>
+      </c>
+      <c r="E98" s="18" t="s">
+        <v>382</v>
+      </c>
+      <c r="F98" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G98" t="s">
+        <v>34</v>
+      </c>
+      <c r="H98" s="18" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="99" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C99" t="s">
+        <v>364</v>
+      </c>
+      <c r="D99" t="s">
+        <v>371</v>
+      </c>
+      <c r="E99" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="F99" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G99" t="s">
+        <v>34</v>
+      </c>
+      <c r="H99" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="J99" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="100" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C100" t="s">
+        <v>364</v>
+      </c>
+      <c r="D100" t="s">
+        <v>372</v>
+      </c>
+      <c r="E100" s="18" t="s">
+        <v>386</v>
+      </c>
+      <c r="F100" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G100" t="s">
+        <v>34</v>
+      </c>
+      <c r="H100" s="18" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="101" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C101" t="s">
+        <v>364</v>
+      </c>
+      <c r="D101" t="s">
+        <v>373</v>
+      </c>
+      <c r="E101" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="F101" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G101" t="s">
+        <v>34</v>
+      </c>
+      <c r="H101" s="18" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="102" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C102" t="s">
+        <v>363</v>
+      </c>
+      <c r="D102" t="s">
+        <v>374</v>
+      </c>
+      <c r="E102" s="18" t="s">
+        <v>390</v>
+      </c>
+      <c r="F102" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G102" t="s">
+        <v>140</v>
+      </c>
+      <c r="H102" s="18" t="s">
+        <v>391</v>
+      </c>
+      <c r="J102" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="103" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C103" t="s">
+        <v>363</v>
+      </c>
+      <c r="D103" t="s">
+        <v>375</v>
+      </c>
+      <c r="E103" s="18" t="s">
+        <v>392</v>
+      </c>
+      <c r="F103" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G103" t="s">
+        <v>140</v>
+      </c>
+      <c r="H103" s="18" t="s">
+        <v>393</v>
+      </c>
+      <c r="J103" t="s">
+        <v>362</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{256F1F5F-11AB-5843-B4A6-909038CC19F4}">
+  <dimension ref="B3:D9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="D3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
+        <v>259</v>
+      </c>
+      <c r="C4" t="s">
+        <v>260</v>
+      </c>
+      <c r="D4" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="C5" t="s">
+        <v>261</v>
+      </c>
+      <c r="D5" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="C6" t="s">
+        <v>262</v>
+      </c>
+      <c r="D6" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>263</v>
+      </c>
+      <c r="C7" t="s">
+        <v>260</v>
+      </c>
+      <c r="D7" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="C8" t="s">
+        <v>261</v>
+      </c>
+      <c r="D8" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="C9" t="s">
+        <v>262</v>
+      </c>
+      <c r="D9" t="s">
+        <v>267</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
0413_Add simulation script for 4-layered hierarchical model (v6)
- Implemented a new R script (simulation_4_layered_v6.R) for simulating data using a 5-layer hierarchical model with an empty 5th layer.
- Defined parameters for binary, continuous, count, and ordinal data types.
- Created functions for sampling positions, generating local positions, and calculating distances.
- Included data generation for each layer and implemented a plotting function for visualizing true positions.
- Added model fitting using the hierarchical LSIRM approach and included diagnostics for acceptance rates and traceplots.
- Implemented distance recovery analysis and position recovery metrics for global and local parameters.
</commit_message>
<xml_diff>
--- a/data/MIDUS_wave_2_변수명세.xlsx
+++ b/data/MIDUS_wave_2_변수명세.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10720"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/todoo/Desktop/학교/대학원/Research/joint_LSIRM/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hyunseokyoon/Desktop/학교/대학원/Research/joint_LSIRM/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8E0F49E-8970-6B4A-AE1A-C5BA2B4B8C4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FADD467E-6846-9044-8C61-72323851E548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="16680" xr2:uid="{D80E1FB4-5E45-DF4A-81BC-88625E0DBDBC}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{D80E1FB4-5E45-DF4A-81BC-88625E0DBDBC}"/>
   </bookViews>
   <sheets>
     <sheet name="wave_2_변수list" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1128" uniqueCount="394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1123" uniqueCount="396">
   <si>
     <t>변수명</t>
   </si>
@@ -1220,6 +1220,12 @@
   </si>
   <si>
     <t>Semantic boundary 통제 실패 / executive monitoring</t>
+  </si>
+  <si>
+    <t>삭제</t>
+  </si>
+  <si>
+    <t>multi 과제 수행 정확성</t>
   </si>
 </sst>
 </file>
@@ -1731,7 +1737,7 @@
     <col min="6" max="6" width="10.1640625" customWidth="1"/>
     <col min="7" max="7" width="18.33203125" customWidth="1"/>
     <col min="8" max="8" width="38.1640625" customWidth="1"/>
-    <col min="9" max="9" width="15.33203125" customWidth="1"/>
+    <col min="9" max="9" width="19.1640625" customWidth="1"/>
     <col min="10" max="10" width="38.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2819,7 +2825,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="54" spans="3:10" x14ac:dyDescent="0.2">
+    <row r="54" spans="3:10" ht="42" x14ac:dyDescent="0.2">
       <c r="C54" s="4" t="s">
         <v>241</v>
       </c>
@@ -2839,7 +2845,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="55" spans="3:10" x14ac:dyDescent="0.2">
+    <row r="55" spans="3:10" ht="42" x14ac:dyDescent="0.2">
       <c r="C55" s="4" t="s">
         <v>241</v>
       </c>
@@ -3550,6 +3556,9 @@
       <c r="H96" s="18" t="s">
         <v>391</v>
       </c>
+      <c r="I96" t="s">
+        <v>394</v>
+      </c>
       <c r="J96" t="s">
         <v>362</v>
       </c>
@@ -3572,6 +3581,9 @@
       </c>
       <c r="H97" s="18" t="s">
         <v>393</v>
+      </c>
+      <c r="I97" t="s">
+        <v>394</v>
       </c>
       <c r="J97" t="s">
         <v>362</v>
@@ -3591,48 +3603,28 @@
       <c r="D100" s="18"/>
       <c r="F100" s="18"/>
       <c r="G100" s="18"/>
+      <c r="H100" s="18" t="s">
+        <v>395</v>
+      </c>
       <c r="I100" s="18"/>
     </row>
     <row r="101" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C101" t="s">
-        <v>363</v>
-      </c>
-      <c r="D101" t="s">
-        <v>358</v>
-      </c>
       <c r="F101" s="18"/>
       <c r="G101" s="18"/>
       <c r="I101" s="18"/>
     </row>
     <row r="102" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C102" t="s">
-        <v>363</v>
-      </c>
-      <c r="D102" t="s">
-        <v>359</v>
-      </c>
       <c r="F102" s="18"/>
       <c r="G102" s="18"/>
+      <c r="H102" s="18"/>
       <c r="I102" s="18"/>
     </row>
     <row r="103" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C103" t="s">
-        <v>365</v>
-      </c>
-      <c r="D103" t="s">
-        <v>351</v>
-      </c>
       <c r="F103" s="18"/>
       <c r="G103" s="18"/>
       <c r="I103" s="18"/>
     </row>
     <row r="104" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C104" t="s">
-        <v>365</v>
-      </c>
-      <c r="D104" t="s">
-        <v>352</v>
-      </c>
       <c r="F104" s="18"/>
       <c r="G104" s="18"/>
       <c r="I104" s="18"/>

</xml_diff>

<commit_message>
0420_add variable, kmeans clustering, comparing with unilayered LSIRM.
</commit_message>
<xml_diff>
--- a/data/MIDUS_wave_2_변수명세.xlsx
+++ b/data/MIDUS_wave_2_변수명세.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hyunseokyoon/Desktop/학교/대학원/Research/joint_LSIRM/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FADD467E-6846-9044-8C61-72323851E548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38C1F943-D2E3-FD45-8C27-D94455E61ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{D80E1FB4-5E45-DF4A-81BC-88625E0DBDBC}"/>
+    <workbookView xWindow="-19200" yWindow="-1860" windowWidth="19200" windowHeight="20980" xr2:uid="{D80E1FB4-5E45-DF4A-81BC-88625E0DBDBC}"/>
   </bookViews>
   <sheets>
     <sheet name="wave_2_변수list" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1123" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1245" uniqueCount="427">
   <si>
     <t>변수명</t>
   </si>
@@ -1072,15 +1072,6 @@
     <t>RA4Q1BBB</t>
   </si>
   <si>
-    <t>wave 2 에는 있으나 refresher 에는 없음</t>
-  </si>
-  <si>
-    <t>wave 2 와 refresher 에 표기가 다름</t>
-  </si>
-  <si>
-    <t>오류 - wave 2 포함해서 확인 필요</t>
-  </si>
-  <si>
     <t>제거 - refresher_1 에 없음</t>
   </si>
   <si>
@@ -1093,139 +1084,571 @@
     <t>RA4H49</t>
   </si>
   <si>
-    <t>B3TSPN</t>
-  </si>
-  <si>
-    <t>B3TSPR</t>
-  </si>
-  <si>
-    <t>B3TSMN</t>
-  </si>
-  <si>
-    <t>B3TSMR</t>
-  </si>
-  <si>
-    <t>B3TSMXBS</t>
-  </si>
-  <si>
-    <t>B3TSMXNO</t>
-  </si>
-  <si>
-    <t>B3TSMXRO</t>
-  </si>
-  <si>
-    <t>B3TCTFLR</t>
-  </si>
-  <si>
-    <t>B3TCTFLI</t>
-  </si>
-  <si>
-    <t>0.5로 나눠서 integer 화 / 문제 상한 20이므로 reverse coding 으로 틀린 문제 수로 해석</t>
-  </si>
-  <si>
-    <t>B3TSMXNS, B3TSMXRS 의 상위지표로 두개 대체 가능</t>
-  </si>
-  <si>
-    <t>zero - inflated 가능성</t>
-  </si>
-  <si>
-    <t>Verbal Fluency</t>
-  </si>
-  <si>
-    <t>Task Switching</t>
-  </si>
-  <si>
-    <t>Executive Function / Processing Speed</t>
-  </si>
-  <si>
     <t>보류(패턴을 해침)</t>
   </si>
   <si>
-    <t>RA3TSPN</t>
-  </si>
-  <si>
-    <t>RA3TSPR</t>
-  </si>
-  <si>
-    <t>RA3TSMN</t>
-  </si>
-  <si>
-    <t>RA3TSMR</t>
-  </si>
-  <si>
-    <t>RA3TSMXBS</t>
-  </si>
-  <si>
-    <t>RA3TSMXNO</t>
-  </si>
-  <si>
-    <t>RA3TSMXRO</t>
-  </si>
-  <si>
-    <t>RA3TCTFLR</t>
-  </si>
-  <si>
-    <t>RA3TCTFLI</t>
-  </si>
-  <si>
-    <t>SGST Normal single-task 정확도 (정답 비율, 0~1)</t>
-  </si>
-  <si>
-    <t>기본 과제 수행 정확성</t>
-  </si>
-  <si>
-    <t>SGST Reverse single-task 정확도 (정답 비율, 0~1)</t>
-  </si>
-  <si>
-    <t>역규칙 과제 수행 정확성 (inhibitory control)</t>
-  </si>
-  <si>
-    <t>SGST Normal single-task 정답 trial median RT (초)</t>
-  </si>
-  <si>
-    <t>기본 인지 처리 속도 baseline</t>
-  </si>
-  <si>
-    <t>SGST Reverse single-task 정답 trial median RT (초)</t>
-  </si>
-  <si>
-    <t>역규칙 처리 속도 (inhibition cost 반영)</t>
-  </si>
-  <si>
-    <t>SGST Mixed block 전체 switch trial median RT (초)</t>
-  </si>
-  <si>
-    <t>규칙 전환 시 반응 속도 (cognitive flexibility)</t>
-  </si>
-  <si>
-    <t>SGST Mixed block normal non-switch trial median RT (초)</t>
-  </si>
-  <si>
-    <t>Mixed block 내 규칙 유지 속도 (normal, mixing cost 포함)</t>
-  </si>
-  <si>
-    <t>SGST Mixed block reverse non-switch trial median RT (초)</t>
-  </si>
-  <si>
-    <t>Mixed block 내 규칙 유지 속도 (reverse, mixing cost 포함)</t>
-  </si>
-  <si>
-    <t>Category fluency 반복 수 (같은 단어 재언급 횟수)</t>
-  </si>
-  <si>
-    <t>자기 모니터링 실패 빈도</t>
-  </si>
-  <si>
-    <t>Category fluency 침입 오류 수 (범주 밖 단어 응답 횟수)</t>
-  </si>
-  <si>
-    <t>Semantic boundary 통제 실패 / executive monitoring</t>
-  </si>
-  <si>
-    <t>삭제</t>
-  </si>
-  <si>
-    <t>multi 과제 수행 정확성</t>
+    <t>cognitive score</t>
+  </si>
+  <si>
+    <t>wl_immediate_omit</t>
+  </si>
+  <si>
+    <t>즉시회상 누락 수 = 15 - 즉시회상 고유회상수</t>
+  </si>
+  <si>
+    <t>M2P3 (ICPSR)</t>
+  </si>
+  <si>
+    <t>즉시 일화기억 저하</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">원변수: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>B3TWLITU</t>
+    </r>
+  </si>
+  <si>
+    <t>wl_immediate_repetition</t>
+  </si>
+  <si>
+    <t>즉시회상 반복 수</t>
+  </si>
+  <si>
+    <t>즉시회상 오류</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">원변수: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>B3TWLITR</t>
+    </r>
+  </si>
+  <si>
+    <t>wl_immediate_intrusion</t>
+  </si>
+  <si>
+    <t>즉시회상 intrusion 수</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">원변수: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>B3TWLITI</t>
+    </r>
+  </si>
+  <si>
+    <t>wl_delayed_omit</t>
+  </si>
+  <si>
+    <t>지연회상 누락 수 = 15 - 지연회상 고유회상수</t>
+  </si>
+  <si>
+    <t>지연 일화기억 저하</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">원변수: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>B3TWLDTU</t>
+    </r>
+  </si>
+  <si>
+    <t>wl_delayed_repetition</t>
+  </si>
+  <si>
+    <t>지연회상 반복 수</t>
+  </si>
+  <si>
+    <t>지연회상 오류</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">원변수: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>B3TWLDTR</t>
+    </r>
+  </si>
+  <si>
+    <t>wl_delayed_intrusion</t>
+  </si>
+  <si>
+    <t>지연회상 intrusion 수</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">원변수: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>B3TWLDTI</t>
+    </r>
+  </si>
+  <si>
+    <t>category fluency</t>
+  </si>
+  <si>
+    <t>catflu_repetition</t>
+  </si>
+  <si>
+    <t>범주유창성 반복 수</t>
+  </si>
+  <si>
+    <t>의미유창성 오류</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">원변수: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>B3TCTFLR</t>
+    </r>
+  </si>
+  <si>
+    <t>catflu_intrusion</t>
+  </si>
+  <si>
+    <t>범주유창성 intrusion 수</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">원변수: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>B3TCTFLI</t>
+    </r>
+  </si>
+  <si>
+    <t>reasoning</t>
+  </si>
+  <si>
+    <t>numseries_incorrect</t>
+  </si>
+  <si>
+    <t>Number Series 오답 수 = 5 - 총정답수</t>
+  </si>
+  <si>
+    <t>귀납추론 저하</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">원변수: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>B3TNSTOT</t>
+    </r>
+  </si>
+  <si>
+    <t>attention / speed</t>
+  </si>
+  <si>
+    <t>backcount_error</t>
+  </si>
+  <si>
+    <t>Backward Counting 오류 수</t>
+  </si>
+  <si>
+    <t>주의·처리속도 오류</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">원변수: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>B3TBKERR</t>
+    </r>
+  </si>
+  <si>
+    <t>executive function / set-shifting</t>
+  </si>
+  <si>
+    <t>sgst_normal_incorrect</t>
+  </si>
+  <si>
+    <t>SGST normal single-task 비정답 수 = 20 - 정답수</t>
+  </si>
+  <si>
+    <t>baseline 실행기능 오류</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">원변수: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>B3TSTN</t>
+    </r>
+  </si>
+  <si>
+    <t>sgst_reverse_incorrect</t>
+  </si>
+  <si>
+    <t>SGST reverse single-task 비정답 수 = 20 - 정답수</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">원변수: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>B3TSTR</t>
+    </r>
+  </si>
+  <si>
+    <t>sgst_mixed_nonswitch_incorrect</t>
+  </si>
+  <si>
+    <t>SGST mixed-task nonswitch 비정답 수 = 23 - 정답수</t>
+  </si>
+  <si>
+    <t>전환 없는 mixed-task 오류</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">원변수: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>B3TSTXBO</t>
+    </r>
+  </si>
+  <si>
+    <t>sgst_mixed_switch_incorrect</t>
+  </si>
+  <si>
+    <t>SGST mixed-task switch 비정답 수 = 6 - 정답수</t>
+  </si>
+  <si>
+    <t>과제전환 오류</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">원변수: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>B3TSTXBS</t>
+    </r>
+  </si>
+  <si>
+    <t>sgst_mixed_all_incorrect</t>
+  </si>
+  <si>
+    <t>SGST mixed-task 전체 비정답 수 = 29 - 정답수</t>
+  </si>
+  <si>
+    <t>전체 전환과제 오류</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">원변수: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>B3TSTXBB</t>
+    </r>
+  </si>
+  <si>
+    <t>제거 여부</t>
+  </si>
+  <si>
+    <r>
+      <t>원변수: RA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>3TWLITU</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>원변수: RA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>3TWLITR</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>원변수: RA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>3TWLITI</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>원변수: RA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>3TWLDTU</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>원변수: RA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>3TWLDTR</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>원변수: RA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>3TWLDTI</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>원변수: RA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>3TCTFLR</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>원변수: RA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>3TCTFLI</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>원변수: RA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>3TNSTOT</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>원변수: RA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>3TBKERR</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>원변수: RA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>3TSTN</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>원변수: RA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>3TSTR</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>원변수: RA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>3TSTXBO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>원변수: RA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>3TSTXBS</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>원변수: RA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>3TSTXBB</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1294,20 +1717,19 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="10"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Arial Unicode MS"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1333,12 +1755,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1370,7 +1786,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1389,9 +1805,6 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -1728,7 +2141,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87BBB518-99D5-8443-BE8B-68691D1BDDA9}">
-  <dimension ref="C3:K108"/>
+  <dimension ref="C3:K102"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="32.5" customWidth="1"/>
@@ -1766,7 +2179,7 @@
         <v>42</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>162</v>
+        <v>411</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>163</v>
@@ -1911,6 +2324,9 @@
       <c r="H11" t="s">
         <v>7</v>
       </c>
+      <c r="I11" t="s">
+        <v>348</v>
+      </c>
     </row>
     <row r="12" spans="3:11" x14ac:dyDescent="0.2">
       <c r="C12" t="s">
@@ -1931,6 +2347,9 @@
       <c r="H12" t="s">
         <v>7</v>
       </c>
+      <c r="I12" t="s">
+        <v>348</v>
+      </c>
     </row>
     <row r="13" spans="3:11" x14ac:dyDescent="0.2">
       <c r="C13" t="s">
@@ -1952,7 +2371,7 @@
         <v>63</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
     </row>
     <row r="14" spans="3:11" x14ac:dyDescent="0.2">
@@ -2014,6 +2433,9 @@
       <c r="H16" t="s">
         <v>41</v>
       </c>
+      <c r="I16" t="s">
+        <v>348</v>
+      </c>
       <c r="K16" s="3"/>
     </row>
     <row r="17" spans="3:9" x14ac:dyDescent="0.2">
@@ -2035,6 +2457,9 @@
       <c r="H17" t="s">
         <v>20</v>
       </c>
+      <c r="I17" t="s">
+        <v>348</v>
+      </c>
     </row>
     <row r="18" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C18" t="s">
@@ -2055,6 +2480,9 @@
       <c r="H18" t="s">
         <v>23</v>
       </c>
+      <c r="I18" t="s">
+        <v>348</v>
+      </c>
     </row>
     <row r="19" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C19" t="s">
@@ -2075,6 +2503,9 @@
       <c r="H19" t="s">
         <v>26</v>
       </c>
+      <c r="I19" t="s">
+        <v>348</v>
+      </c>
     </row>
     <row r="20" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C20" t="s">
@@ -2095,6 +2526,9 @@
       <c r="H20" t="s">
         <v>71</v>
       </c>
+      <c r="I20" t="s">
+        <v>348</v>
+      </c>
     </row>
     <row r="21" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C21" t="s">
@@ -2115,6 +2549,9 @@
       <c r="H21" t="s">
         <v>71</v>
       </c>
+      <c r="I21" t="s">
+        <v>348</v>
+      </c>
     </row>
     <row r="22" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C22" t="s">
@@ -2136,7 +2573,7 @@
         <v>75</v>
       </c>
       <c r="I22" t="s">
-        <v>366</v>
+        <v>348</v>
       </c>
     </row>
     <row r="23" spans="3:9" x14ac:dyDescent="0.2">
@@ -2159,7 +2596,7 @@
         <v>76</v>
       </c>
       <c r="I23" t="s">
-        <v>366</v>
+        <v>348</v>
       </c>
     </row>
     <row r="24" spans="3:9" x14ac:dyDescent="0.2">
@@ -2242,7 +2679,7 @@
         <v>147</v>
       </c>
       <c r="I27" t="s">
-        <v>366</v>
+        <v>348</v>
       </c>
     </row>
     <row r="28" spans="3:9" x14ac:dyDescent="0.2">
@@ -2265,7 +2702,7 @@
         <v>151</v>
       </c>
       <c r="I28" t="s">
-        <v>366</v>
+        <v>348</v>
       </c>
     </row>
     <row r="29" spans="3:9" x14ac:dyDescent="0.2">
@@ -2288,7 +2725,7 @@
         <v>155</v>
       </c>
       <c r="I29" t="s">
-        <v>366</v>
+        <v>348</v>
       </c>
     </row>
     <row r="30" spans="3:9" x14ac:dyDescent="0.2">
@@ -2311,7 +2748,7 @@
         <v>159</v>
       </c>
       <c r="I30" t="s">
-        <v>366</v>
+        <v>348</v>
       </c>
     </row>
     <row r="31" spans="3:9" x14ac:dyDescent="0.2">
@@ -3387,275 +3824,395 @@
     </row>
     <row r="82" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="83" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="84" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="89" spans="3:10" x14ac:dyDescent="0.2">
+    <row r="84" spans="3:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C84" t="s">
+        <v>349</v>
+      </c>
+      <c r="F84" s="14"/>
+      <c r="G84" s="14"/>
+      <c r="I84" s="14"/>
+    </row>
+    <row r="85" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C85" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H85" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="I85" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="J85" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="86" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C86" t="s">
+        <v>67</v>
+      </c>
+      <c r="D86" s="15" t="s">
+        <v>350</v>
+      </c>
+      <c r="E86" t="s">
+        <v>351</v>
+      </c>
+      <c r="F86" t="s">
+        <v>352</v>
+      </c>
+      <c r="G86" t="s">
+        <v>140</v>
+      </c>
+      <c r="H86" t="s">
+        <v>353</v>
+      </c>
+      <c r="J86" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="87" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C87" t="s">
+        <v>67</v>
+      </c>
+      <c r="D87" s="15" t="s">
+        <v>355</v>
+      </c>
+      <c r="E87" t="s">
+        <v>356</v>
+      </c>
+      <c r="F87" t="s">
+        <v>352</v>
+      </c>
+      <c r="G87" t="s">
+        <v>140</v>
+      </c>
+      <c r="H87" t="s">
+        <v>357</v>
+      </c>
+      <c r="J87" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="88" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C88" t="s">
+        <v>67</v>
+      </c>
+      <c r="D88" s="15" t="s">
+        <v>359</v>
+      </c>
+      <c r="E88" t="s">
+        <v>360</v>
+      </c>
+      <c r="F88" t="s">
+        <v>352</v>
+      </c>
+      <c r="G88" t="s">
+        <v>140</v>
+      </c>
+      <c r="H88" t="s">
+        <v>357</v>
+      </c>
+      <c r="J88" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="89" spans="3:10" ht="17" x14ac:dyDescent="0.25">
       <c r="C89" t="s">
-        <v>365</v>
-      </c>
-      <c r="D89" t="s">
-        <v>351</v>
-      </c>
-      <c r="E89" s="18" t="s">
-        <v>376</v>
-      </c>
-      <c r="F89" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
+      </c>
+      <c r="D89" s="15" t="s">
+        <v>362</v>
+      </c>
+      <c r="E89" t="s">
+        <v>363</v>
+      </c>
+      <c r="F89" t="s">
+        <v>352</v>
       </c>
       <c r="G89" t="s">
         <v>140</v>
       </c>
-      <c r="H89" s="18" t="s">
-        <v>377</v>
+      <c r="H89" t="s">
+        <v>364</v>
       </c>
       <c r="J89" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="90" spans="3:10" x14ac:dyDescent="0.2">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="90" spans="3:10" ht="17" x14ac:dyDescent="0.25">
       <c r="C90" t="s">
-        <v>365</v>
-      </c>
-      <c r="D90" t="s">
+        <v>67</v>
+      </c>
+      <c r="D90" s="15" t="s">
+        <v>366</v>
+      </c>
+      <c r="E90" t="s">
+        <v>367</v>
+      </c>
+      <c r="F90" t="s">
         <v>352</v>
-      </c>
-      <c r="E90" s="18" t="s">
-        <v>378</v>
-      </c>
-      <c r="F90" s="1" t="s">
-        <v>66</v>
       </c>
       <c r="G90" t="s">
         <v>140</v>
       </c>
-      <c r="H90" s="18" t="s">
+      <c r="H90" t="s">
+        <v>368</v>
+      </c>
+      <c r="J90" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="91" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C91" t="s">
+        <v>67</v>
+      </c>
+      <c r="D91" s="15" t="s">
+        <v>370</v>
+      </c>
+      <c r="E91" t="s">
+        <v>371</v>
+      </c>
+      <c r="F91" t="s">
+        <v>352</v>
+      </c>
+      <c r="G91" t="s">
+        <v>140</v>
+      </c>
+      <c r="H91" t="s">
+        <v>368</v>
+      </c>
+      <c r="J91" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="92" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C92" t="s">
+        <v>373</v>
+      </c>
+      <c r="D92" s="15" t="s">
+        <v>374</v>
+      </c>
+      <c r="E92" t="s">
+        <v>375</v>
+      </c>
+      <c r="F92" t="s">
+        <v>352</v>
+      </c>
+      <c r="G92" t="s">
+        <v>140</v>
+      </c>
+      <c r="H92" t="s">
+        <v>376</v>
+      </c>
+      <c r="J92" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="93" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C93" t="s">
+        <v>373</v>
+      </c>
+      <c r="D93" s="15" t="s">
+        <v>378</v>
+      </c>
+      <c r="E93" t="s">
         <v>379</v>
       </c>
-      <c r="J90" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="91" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C91" t="s">
-        <v>365</v>
-      </c>
-      <c r="D91" t="s">
-        <v>353</v>
-      </c>
-      <c r="E91" s="18" t="s">
+      <c r="F93" t="s">
+        <v>352</v>
+      </c>
+      <c r="G93" t="s">
+        <v>140</v>
+      </c>
+      <c r="H93" t="s">
+        <v>376</v>
+      </c>
+      <c r="J93" t="s">
         <v>380</v>
       </c>
-      <c r="F91" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G91" t="s">
-        <v>34</v>
-      </c>
-      <c r="H91" s="18" t="s">
+    </row>
+    <row r="94" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C94" t="s">
         <v>381</v>
       </c>
-    </row>
-    <row r="92" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C92" t="s">
-        <v>365</v>
-      </c>
-      <c r="D92" t="s">
-        <v>354</v>
-      </c>
-      <c r="E92" s="18" t="s">
+      <c r="D94" s="15" t="s">
         <v>382</v>
       </c>
-      <c r="F92" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G92" t="s">
-        <v>34</v>
-      </c>
-      <c r="H92" s="18" t="s">
+      <c r="E94" t="s">
         <v>383</v>
       </c>
-    </row>
-    <row r="93" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C93" t="s">
-        <v>364</v>
-      </c>
-      <c r="D93" t="s">
-        <v>355</v>
-      </c>
-      <c r="E93" s="18" t="s">
+      <c r="F94" t="s">
+        <v>352</v>
+      </c>
+      <c r="G94" t="s">
+        <v>140</v>
+      </c>
+      <c r="H94" t="s">
         <v>384</v>
       </c>
-      <c r="F93" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G93" t="s">
-        <v>34</v>
-      </c>
-      <c r="H93" s="18" t="s">
+      <c r="J94" t="s">
         <v>385</v>
       </c>
-      <c r="J93" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="94" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C94" t="s">
-        <v>364</v>
-      </c>
-      <c r="D94" t="s">
-        <v>356</v>
-      </c>
-      <c r="E94" s="18" t="s">
+    </row>
+    <row r="95" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C95" t="s">
         <v>386</v>
       </c>
-      <c r="F94" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G94" t="s">
-        <v>34</v>
-      </c>
-      <c r="H94" s="18" t="s">
+      <c r="D95" s="15" t="s">
         <v>387</v>
       </c>
-    </row>
-    <row r="95" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C95" t="s">
-        <v>364</v>
-      </c>
-      <c r="D95" t="s">
-        <v>357</v>
-      </c>
-      <c r="E95" s="18" t="s">
+      <c r="E95" t="s">
         <v>388</v>
       </c>
-      <c r="F95" s="1" t="s">
-        <v>66</v>
+      <c r="F95" t="s">
+        <v>352</v>
       </c>
       <c r="G95" t="s">
-        <v>34</v>
-      </c>
-      <c r="H95" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="H95" t="s">
         <v>389</v>
       </c>
-    </row>
-    <row r="96" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="J95" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="96" spans="3:10" ht="17" x14ac:dyDescent="0.25">
       <c r="C96" t="s">
-        <v>363</v>
-      </c>
-      <c r="D96" t="s">
-        <v>358</v>
-      </c>
-      <c r="E96" s="18" t="s">
-        <v>390</v>
-      </c>
-      <c r="F96" s="1" t="s">
-        <v>66</v>
+        <v>391</v>
+      </c>
+      <c r="D96" s="15" t="s">
+        <v>392</v>
+      </c>
+      <c r="E96" t="s">
+        <v>393</v>
+      </c>
+      <c r="F96" t="s">
+        <v>352</v>
       </c>
       <c r="G96" t="s">
         <v>140</v>
       </c>
-      <c r="H96" s="18" t="s">
+      <c r="H96" t="s">
+        <v>394</v>
+      </c>
+      <c r="J96" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="97" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C97" t="s">
         <v>391</v>
       </c>
-      <c r="I96" t="s">
-        <v>394</v>
-      </c>
-      <c r="J96" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="97" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C97" t="s">
-        <v>363</v>
-      </c>
-      <c r="D97" t="s">
-        <v>359</v>
-      </c>
-      <c r="E97" s="18" t="s">
-        <v>392</v>
-      </c>
-      <c r="F97" s="1" t="s">
-        <v>66</v>
+      <c r="D97" s="15" t="s">
+        <v>396</v>
+      </c>
+      <c r="E97" t="s">
+        <v>397</v>
+      </c>
+      <c r="F97" t="s">
+        <v>352</v>
       </c>
       <c r="G97" t="s">
         <v>140</v>
       </c>
-      <c r="H97" s="18" t="s">
-        <v>393</v>
-      </c>
-      <c r="I97" t="s">
+      <c r="H97" t="s">
         <v>394</v>
       </c>
       <c r="J97" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="99" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C99" s="17"/>
-      <c r="D99" s="17"/>
-      <c r="E99" s="17"/>
-      <c r="F99" s="17"/>
-      <c r="G99" s="17"/>
-      <c r="H99" s="17"/>
-      <c r="I99" s="17"/>
-    </row>
-    <row r="100" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C100" s="18"/>
-      <c r="D100" s="18"/>
-      <c r="F100" s="18"/>
-      <c r="G100" s="18"/>
-      <c r="H100" s="18" t="s">
-        <v>395</v>
-      </c>
-      <c r="I100" s="18"/>
+        <v>398</v>
+      </c>
+    </row>
+    <row r="98" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C98" t="s">
+        <v>391</v>
+      </c>
+      <c r="D98" s="15" t="s">
+        <v>399</v>
+      </c>
+      <c r="E98" t="s">
+        <v>400</v>
+      </c>
+      <c r="F98" t="s">
+        <v>352</v>
+      </c>
+      <c r="G98" t="s">
+        <v>140</v>
+      </c>
+      <c r="H98" t="s">
+        <v>401</v>
+      </c>
+      <c r="J98" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="99" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C99" t="s">
+        <v>391</v>
+      </c>
+      <c r="D99" s="15" t="s">
+        <v>403</v>
+      </c>
+      <c r="E99" t="s">
+        <v>404</v>
+      </c>
+      <c r="F99" t="s">
+        <v>352</v>
+      </c>
+      <c r="G99" t="s">
+        <v>140</v>
+      </c>
+      <c r="H99" t="s">
+        <v>405</v>
+      </c>
+      <c r="J99" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="100" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C100" t="s">
+        <v>391</v>
+      </c>
+      <c r="D100" s="15" t="s">
+        <v>407</v>
+      </c>
+      <c r="E100" t="s">
+        <v>408</v>
+      </c>
+      <c r="F100" t="s">
+        <v>352</v>
+      </c>
+      <c r="G100" t="s">
+        <v>140</v>
+      </c>
+      <c r="H100" t="s">
+        <v>409</v>
+      </c>
+      <c r="J100" t="s">
+        <v>410</v>
+      </c>
     </row>
     <row r="101" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="F101" s="18"/>
-      <c r="G101" s="18"/>
-      <c r="I101" s="18"/>
+      <c r="F101" s="14"/>
+      <c r="G101" s="14"/>
+      <c r="I101" s="14"/>
     </row>
     <row r="102" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="F102" s="18"/>
-      <c r="G102" s="18"/>
-      <c r="H102" s="18"/>
-      <c r="I102" s="18"/>
-    </row>
-    <row r="103" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="F103" s="18"/>
-      <c r="G103" s="18"/>
-      <c r="I103" s="18"/>
-    </row>
-    <row r="104" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="F104" s="18"/>
-      <c r="G104" s="18"/>
-      <c r="I104" s="18"/>
-    </row>
-    <row r="105" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C105" s="18"/>
-      <c r="D105" s="18"/>
-      <c r="F105" s="18"/>
-      <c r="G105" s="18"/>
-      <c r="I105" s="18"/>
-    </row>
-    <row r="106" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C106" s="18"/>
-      <c r="D106" s="18"/>
-      <c r="F106" s="18"/>
-      <c r="G106" s="18"/>
-      <c r="I106" s="18"/>
-    </row>
-    <row r="107" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C107" s="18"/>
-      <c r="D107" s="18"/>
-      <c r="F107" s="18"/>
-      <c r="G107" s="18"/>
-      <c r="I107" s="18"/>
-    </row>
-    <row r="108" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C108" s="18"/>
-      <c r="D108" s="18"/>
-      <c r="F108" s="18"/>
-      <c r="G108" s="18"/>
-      <c r="I108" s="18"/>
+      <c r="F102" s="14"/>
+      <c r="G102" s="14"/>
+      <c r="H102" s="14"/>
+      <c r="I102" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
@@ -3867,7 +4424,9 @@
       <c r="H11" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I11" s="6"/>
+      <c r="I11" t="s">
+        <v>348</v>
+      </c>
       <c r="J11" s="6"/>
     </row>
     <row r="12" spans="3:10" x14ac:dyDescent="0.2">
@@ -3889,7 +4448,9 @@
       <c r="H12" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I12" s="6"/>
+      <c r="I12" t="s">
+        <v>348</v>
+      </c>
       <c r="J12" s="6"/>
     </row>
     <row r="13" spans="3:10" x14ac:dyDescent="0.2">
@@ -3912,7 +4473,7 @@
         <v>63</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="J13" s="6"/>
     </row>
@@ -3979,7 +4540,9 @@
       <c r="H16" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="I16" s="6"/>
+      <c r="I16" s="6" t="s">
+        <v>348</v>
+      </c>
       <c r="J16" s="6"/>
     </row>
     <row r="17" spans="3:10" x14ac:dyDescent="0.2">
@@ -4001,7 +4564,9 @@
       <c r="H17" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I17" s="6"/>
+      <c r="I17" s="6" t="s">
+        <v>348</v>
+      </c>
       <c r="J17" s="6"/>
     </row>
     <row r="18" spans="3:10" x14ac:dyDescent="0.2">
@@ -4023,7 +4588,9 @@
       <c r="H18" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="I18" s="6"/>
+      <c r="I18" s="6" t="s">
+        <v>348</v>
+      </c>
       <c r="J18" s="6"/>
     </row>
     <row r="19" spans="3:10" x14ac:dyDescent="0.2">
@@ -4045,7 +4612,9 @@
       <c r="H19" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="I19" s="6"/>
+      <c r="I19" s="6" t="s">
+        <v>348</v>
+      </c>
       <c r="J19" s="6"/>
     </row>
     <row r="20" spans="3:10" x14ac:dyDescent="0.2">
@@ -4067,7 +4636,9 @@
       <c r="H20" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="I20" s="6"/>
+      <c r="I20" s="6" t="s">
+        <v>348</v>
+      </c>
       <c r="J20" s="6"/>
     </row>
     <row r="21" spans="3:10" x14ac:dyDescent="0.2">
@@ -4089,7 +4660,9 @@
       <c r="H21" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="I21" s="6"/>
+      <c r="I21" s="6" t="s">
+        <v>348</v>
+      </c>
       <c r="J21" s="6"/>
     </row>
     <row r="22" spans="3:10" x14ac:dyDescent="0.2">
@@ -4111,7 +4684,9 @@
       <c r="H22" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="I22" s="6"/>
+      <c r="I22" s="6" t="s">
+        <v>348</v>
+      </c>
       <c r="J22" s="6"/>
     </row>
     <row r="23" spans="3:10" x14ac:dyDescent="0.2">
@@ -4133,7 +4708,9 @@
       <c r="H23" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="I23" s="6"/>
+      <c r="I23" s="6" t="s">
+        <v>348</v>
+      </c>
       <c r="J23" s="6"/>
     </row>
     <row r="24" spans="3:10" x14ac:dyDescent="0.2">
@@ -4207,7 +4784,7 @@
         <v>144</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>146</v>
@@ -4251,7 +4828,7 @@
         <v>152</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>154</v>
@@ -4273,7 +4850,7 @@
         <v>156</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="E30" s="9" t="s">
         <v>158</v>
@@ -5383,218 +5960,399 @@
         <v>248</v>
       </c>
     </row>
+    <row r="84" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C84" t="s">
+        <v>349</v>
+      </c>
+      <c r="F84" s="14"/>
+      <c r="G84" s="14"/>
+      <c r="I84" s="14"/>
+    </row>
     <row r="85" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C85" s="14"/>
-      <c r="D85" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="86" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C86" s="15"/>
-      <c r="D86" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="87" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C87" s="16"/>
-      <c r="D87" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="95" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C85" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H85" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="I85" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="J85" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="86" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C86" t="s">
+        <v>67</v>
+      </c>
+      <c r="D86" s="15" t="s">
+        <v>350</v>
+      </c>
+      <c r="E86" t="s">
+        <v>351</v>
+      </c>
+      <c r="F86" t="s">
+        <v>352</v>
+      </c>
+      <c r="G86" t="s">
+        <v>140</v>
+      </c>
+      <c r="H86" t="s">
+        <v>353</v>
+      </c>
+      <c r="J86" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="87" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C87" t="s">
+        <v>67</v>
+      </c>
+      <c r="D87" s="15" t="s">
+        <v>355</v>
+      </c>
+      <c r="E87" t="s">
+        <v>356</v>
+      </c>
+      <c r="F87" t="s">
+        <v>352</v>
+      </c>
+      <c r="G87" t="s">
+        <v>140</v>
+      </c>
+      <c r="H87" t="s">
+        <v>357</v>
+      </c>
+      <c r="J87" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="88" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C88" t="s">
+        <v>67</v>
+      </c>
+      <c r="D88" s="15" t="s">
+        <v>359</v>
+      </c>
+      <c r="E88" t="s">
+        <v>360</v>
+      </c>
+      <c r="F88" t="s">
+        <v>352</v>
+      </c>
+      <c r="G88" t="s">
+        <v>140</v>
+      </c>
+      <c r="H88" t="s">
+        <v>357</v>
+      </c>
+      <c r="J88" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="89" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C89" t="s">
+        <v>67</v>
+      </c>
+      <c r="D89" s="15" t="s">
+        <v>362</v>
+      </c>
+      <c r="E89" t="s">
+        <v>363</v>
+      </c>
+      <c r="F89" t="s">
+        <v>352</v>
+      </c>
+      <c r="G89" t="s">
+        <v>140</v>
+      </c>
+      <c r="H89" t="s">
+        <v>364</v>
+      </c>
+      <c r="J89" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="90" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C90" t="s">
+        <v>67</v>
+      </c>
+      <c r="D90" s="15" t="s">
+        <v>366</v>
+      </c>
+      <c r="E90" t="s">
+        <v>367</v>
+      </c>
+      <c r="F90" t="s">
+        <v>352</v>
+      </c>
+      <c r="G90" t="s">
+        <v>140</v>
+      </c>
+      <c r="H90" t="s">
+        <v>368</v>
+      </c>
+      <c r="J90" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="91" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C91" t="s">
+        <v>67</v>
+      </c>
+      <c r="D91" s="15" t="s">
+        <v>370</v>
+      </c>
+      <c r="E91" t="s">
+        <v>371</v>
+      </c>
+      <c r="F91" t="s">
+        <v>352</v>
+      </c>
+      <c r="G91" t="s">
+        <v>140</v>
+      </c>
+      <c r="H91" t="s">
+        <v>368</v>
+      </c>
+      <c r="J91" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="92" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C92" t="s">
+        <v>373</v>
+      </c>
+      <c r="D92" s="15" t="s">
+        <v>374</v>
+      </c>
+      <c r="E92" t="s">
+        <v>375</v>
+      </c>
+      <c r="F92" t="s">
+        <v>352</v>
+      </c>
+      <c r="G92" t="s">
+        <v>140</v>
+      </c>
+      <c r="H92" t="s">
+        <v>376</v>
+      </c>
+      <c r="J92" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="93" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C93" t="s">
+        <v>373</v>
+      </c>
+      <c r="D93" s="15" t="s">
+        <v>378</v>
+      </c>
+      <c r="E93" t="s">
+        <v>379</v>
+      </c>
+      <c r="F93" t="s">
+        <v>352</v>
+      </c>
+      <c r="G93" t="s">
+        <v>140</v>
+      </c>
+      <c r="H93" t="s">
+        <v>376</v>
+      </c>
+      <c r="J93" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="94" spans="3:10" ht="17" x14ac:dyDescent="0.25">
+      <c r="C94" t="s">
+        <v>381</v>
+      </c>
+      <c r="D94" s="15" t="s">
+        <v>382</v>
+      </c>
+      <c r="E94" t="s">
+        <v>383</v>
+      </c>
+      <c r="F94" t="s">
+        <v>352</v>
+      </c>
+      <c r="G94" t="s">
+        <v>140</v>
+      </c>
+      <c r="H94" t="s">
+        <v>384</v>
+      </c>
+      <c r="J94" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="95" spans="3:10" ht="17" x14ac:dyDescent="0.25">
       <c r="C95" t="s">
-        <v>365</v>
-      </c>
-      <c r="D95" t="s">
-        <v>367</v>
-      </c>
-      <c r="E95" s="18" t="s">
-        <v>376</v>
-      </c>
-      <c r="F95" s="7" t="s">
-        <v>272</v>
+        <v>386</v>
+      </c>
+      <c r="D95" s="15" t="s">
+        <v>387</v>
+      </c>
+      <c r="E95" t="s">
+        <v>388</v>
+      </c>
+      <c r="F95" t="s">
+        <v>352</v>
       </c>
       <c r="G95" t="s">
         <v>140</v>
       </c>
-      <c r="H95" s="18" t="s">
-        <v>377</v>
+      <c r="H95" t="s">
+        <v>389</v>
       </c>
       <c r="J95" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="96" spans="3:10" x14ac:dyDescent="0.2">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="96" spans="3:10" ht="17" x14ac:dyDescent="0.25">
       <c r="C96" t="s">
-        <v>365</v>
-      </c>
-      <c r="D96" t="s">
-        <v>368</v>
-      </c>
-      <c r="E96" s="18" t="s">
-        <v>378</v>
-      </c>
-      <c r="F96" s="7" t="s">
-        <v>272</v>
+        <v>391</v>
+      </c>
+      <c r="D96" s="15" t="s">
+        <v>392</v>
+      </c>
+      <c r="E96" t="s">
+        <v>393</v>
+      </c>
+      <c r="F96" t="s">
+        <v>352</v>
       </c>
       <c r="G96" t="s">
         <v>140</v>
       </c>
-      <c r="H96" s="18" t="s">
-        <v>379</v>
+      <c r="H96" t="s">
+        <v>394</v>
       </c>
       <c r="J96" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="97" spans="3:10" x14ac:dyDescent="0.2">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="97" spans="3:10" ht="17" x14ac:dyDescent="0.25">
       <c r="C97" t="s">
-        <v>365</v>
-      </c>
-      <c r="D97" t="s">
-        <v>369</v>
-      </c>
-      <c r="E97" s="18" t="s">
-        <v>380</v>
-      </c>
-      <c r="F97" s="7" t="s">
-        <v>272</v>
+        <v>391</v>
+      </c>
+      <c r="D97" s="15" t="s">
+        <v>396</v>
+      </c>
+      <c r="E97" t="s">
+        <v>397</v>
+      </c>
+      <c r="F97" t="s">
+        <v>352</v>
       </c>
       <c r="G97" t="s">
-        <v>34</v>
-      </c>
-      <c r="H97" s="18" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="98" spans="3:10" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+      <c r="H97" t="s">
+        <v>394</v>
+      </c>
+      <c r="J97" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="98" spans="3:10" ht="17" x14ac:dyDescent="0.25">
       <c r="C98" t="s">
-        <v>365</v>
-      </c>
-      <c r="D98" t="s">
-        <v>370</v>
-      </c>
-      <c r="E98" s="18" t="s">
-        <v>382</v>
-      </c>
-      <c r="F98" s="7" t="s">
-        <v>272</v>
+        <v>391</v>
+      </c>
+      <c r="D98" s="15" t="s">
+        <v>399</v>
+      </c>
+      <c r="E98" t="s">
+        <v>400</v>
+      </c>
+      <c r="F98" t="s">
+        <v>352</v>
       </c>
       <c r="G98" t="s">
-        <v>34</v>
-      </c>
-      <c r="H98" s="18" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="99" spans="3:10" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+      <c r="H98" t="s">
+        <v>401</v>
+      </c>
+      <c r="J98" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="99" spans="3:10" ht="17" x14ac:dyDescent="0.25">
       <c r="C99" t="s">
-        <v>364</v>
-      </c>
-      <c r="D99" t="s">
-        <v>371</v>
-      </c>
-      <c r="E99" s="18" t="s">
-        <v>384</v>
-      </c>
-      <c r="F99" s="7" t="s">
-        <v>272</v>
+        <v>391</v>
+      </c>
+      <c r="D99" s="15" t="s">
+        <v>403</v>
+      </c>
+      <c r="E99" t="s">
+        <v>404</v>
+      </c>
+      <c r="F99" t="s">
+        <v>352</v>
       </c>
       <c r="G99" t="s">
-        <v>34</v>
-      </c>
-      <c r="H99" s="18" t="s">
-        <v>385</v>
+        <v>140</v>
+      </c>
+      <c r="H99" t="s">
+        <v>405</v>
       </c>
       <c r="J99" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="100" spans="3:10" x14ac:dyDescent="0.2">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="100" spans="3:10" ht="17" x14ac:dyDescent="0.25">
       <c r="C100" t="s">
-        <v>364</v>
-      </c>
-      <c r="D100" t="s">
-        <v>372</v>
-      </c>
-      <c r="E100" s="18" t="s">
-        <v>386</v>
-      </c>
-      <c r="F100" s="7" t="s">
-        <v>272</v>
+        <v>391</v>
+      </c>
+      <c r="D100" s="15" t="s">
+        <v>407</v>
+      </c>
+      <c r="E100" t="s">
+        <v>408</v>
+      </c>
+      <c r="F100" t="s">
+        <v>352</v>
       </c>
       <c r="G100" t="s">
-        <v>34</v>
-      </c>
-      <c r="H100" s="18" t="s">
-        <v>387</v>
+        <v>140</v>
+      </c>
+      <c r="H100" t="s">
+        <v>409</v>
+      </c>
+      <c r="J100" t="s">
+        <v>426</v>
       </c>
     </row>
     <row r="101" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C101" t="s">
-        <v>364</v>
-      </c>
-      <c r="D101" t="s">
-        <v>373</v>
-      </c>
-      <c r="E101" s="18" t="s">
-        <v>388</v>
-      </c>
-      <c r="F101" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="G101" t="s">
-        <v>34</v>
-      </c>
-      <c r="H101" s="18" t="s">
-        <v>389</v>
-      </c>
+      <c r="E101" s="14"/>
+      <c r="F101" s="7"/>
+      <c r="H101" s="14"/>
     </row>
     <row r="102" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C102" t="s">
-        <v>363</v>
-      </c>
-      <c r="D102" t="s">
-        <v>374</v>
-      </c>
-      <c r="E102" s="18" t="s">
-        <v>390</v>
-      </c>
-      <c r="F102" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="G102" t="s">
-        <v>140</v>
-      </c>
-      <c r="H102" s="18" t="s">
-        <v>391</v>
-      </c>
-      <c r="J102" t="s">
-        <v>362</v>
-      </c>
+      <c r="E102" s="14"/>
+      <c r="F102" s="7"/>
+      <c r="H102" s="14"/>
     </row>
     <row r="103" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C103" t="s">
-        <v>363</v>
-      </c>
-      <c r="D103" t="s">
-        <v>375</v>
-      </c>
-      <c r="E103" s="18" t="s">
-        <v>392</v>
-      </c>
-      <c r="F103" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="G103" t="s">
-        <v>140</v>
-      </c>
-      <c r="H103" s="18" t="s">
-        <v>393</v>
-      </c>
-      <c r="J103" t="s">
-        <v>362</v>
-      </c>
+      <c r="E103" s="14"/>
+      <c r="F103" s="7"/>
+      <c r="H103" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>